<commit_message>
Inventory functionality is running successfully
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -18,7 +18,7 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="360">
   <si>
     <t>Sauce Demo Test Scenario</t>
   </si>
@@ -1047,12 +1047,103 @@
   </si>
   <si>
     <t>LOCKED_USER</t>
+  </si>
+  <si>
+    <t>$29.99</t>
+  </si>
+  <si>
+    <t>carry.allTheThings() with the sleek, streamlined Sly Pack that melds uncompromising style with unequaled laptop and tablet protection.</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/static/media/sauce-backpack-1200x1500.0a0b85a385945026062b.jpg</t>
+  </si>
+  <si>
+    <t>01-07-2026 15:38:47</t>
+  </si>
+  <si>
+    <t>chrome</t>
+  </si>
+  <si>
+    <t>Sauce Labs Bike Light</t>
+  </si>
+  <si>
+    <t>$9.99</t>
+  </si>
+  <si>
+    <t>A red light isn't the desired state in testing but it sure helps when riding your bike at night. Water-resistant with 3 lighting modes, 1 AAA battery included.</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/static/media/bike-light-1200x1500.37c843b09a7d77409d63.jpg</t>
+  </si>
+  <si>
+    <t>Sauce Labs Bolt T-Shirt</t>
+  </si>
+  <si>
+    <t>$15.99</t>
+  </si>
+  <si>
+    <t>Get your testing superhero on with the Sauce Labs bolt T-shirt. From American Apparel, 100% ringspun combed cotton, heather gray with red bolt.</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/static/media/bolt-shirt-1200x1500.c2599ac5f0a35ed5931e.jpg</t>
+  </si>
+  <si>
+    <t>Sauce Labs Fleece Jacket</t>
+  </si>
+  <si>
+    <t>$49.99</t>
+  </si>
+  <si>
+    <t>It's not every day that you come across a midweight quarter-zip fleece jacket capable of handling everything from a relaxing day outdoors to a busy day at the office.</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/static/media/sauce-pullover-1200x1500.51d7ffaf301e698772c8.jpg</t>
+  </si>
+  <si>
+    <t>Sauce Labs Onesie</t>
+  </si>
+  <si>
+    <t>$7.99</t>
+  </si>
+  <si>
+    <t>Rib snap infant onesie for the junior automation engineer in development. Reinforced 3-snap bottom closure, two-needle hemmed sleeved and bottom won't unravel.</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/static/media/red-onesie-1200x1500.2ec615b271ef4c3bc430.jpg</t>
+  </si>
+  <si>
+    <t>Test.allTheThings() T-Shirt (Red)</t>
+  </si>
+  <si>
+    <t>This classic Sauce Labs t-shirt is perfect to wear when cozying up to your keyboard to automate a few tests. Super-soft and comfy ringspun combed cotton.</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/static/media/red-tatt-1200x1500.30dadef477804e54fc7b.jpg</t>
+  </si>
+  <si>
+    <t>Sauce Labs Backpack - $29.99</t>
+  </si>
+  <si>
+    <t>Sauce Labs Bike Light - $9.99</t>
+  </si>
+  <si>
+    <t>Sauce Labs Bolt T-Shirt - $15.99</t>
+  </si>
+  <si>
+    <t>Sauce Labs Fleece Jacket - $49.99</t>
+  </si>
+  <si>
+    <t>Sauce Labs Onesie - $7.99</t>
+  </si>
+  <si>
+    <t>Test.allTheThings() T-Shirt (Red) - $15.99</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="8">
     <font>
       <sz val="11"/>
@@ -2134,11 +2225,11 @@
   <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="35.25" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="50" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" customWidth="true" style="1" width="16.5703125"/>
+    <col min="2" max="2" customWidth="true" style="1" width="22.140625"/>
+    <col min="3" max="3" customWidth="true" style="2" width="50.0"/>
+    <col min="4" max="4" customWidth="true" style="1" width="18.0"/>
+    <col min="5" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="35.25" customHeight="1">
@@ -2481,15 +2572,15 @@
   <dimension ref="A1:I62"/>
   <sheetFormatPr defaultRowHeight="35.25" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" style="43" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="28.140625" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="29" customWidth="1"/>
-    <col min="6" max="6" width="32.5703125" customWidth="1"/>
-    <col min="7" max="7" width="35.28515625" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" customWidth="1"/>
-    <col min="9" max="9" width="23.28515625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" style="43" width="20.28515625"/>
+    <col min="2" max="2" customWidth="true" style="6" width="19.5703125"/>
+    <col min="3" max="3" customWidth="true" width="28.140625"/>
+    <col min="4" max="4" customWidth="true" width="20.7109375"/>
+    <col min="5" max="5" customWidth="true" width="29.0"/>
+    <col min="6" max="6" customWidth="true" width="32.5703125"/>
+    <col min="7" max="7" customWidth="true" width="35.28515625"/>
+    <col min="8" max="8" customWidth="true" width="18.7109375"/>
+    <col min="9" max="9" customWidth="true" width="23.28515625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="35.25" customHeight="1">
@@ -3886,20 +3977,20 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35697644-06C4-4BF4-833F-2719491F902D}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" style="57" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" style="57" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" style="57" customWidth="1"/>
-    <col min="4" max="4" width="16" style="57" customWidth="1"/>
-    <col min="5" max="5" width="19.28515625" style="57" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" style="57" customWidth="1"/>
-    <col min="7" max="7" width="19" style="57" customWidth="1"/>
-    <col min="8" max="8" width="18.5703125" style="57" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" style="57" customWidth="1"/>
-    <col min="10" max="10" width="12.42578125" style="57" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="57"/>
+    <col min="1" max="1" customWidth="true" style="57" width="17.42578125"/>
+    <col min="2" max="2" customWidth="true" style="57" width="18.5703125"/>
+    <col min="3" max="3" customWidth="true" style="57" width="17.42578125"/>
+    <col min="4" max="4" customWidth="true" style="57" width="16.0"/>
+    <col min="5" max="5" customWidth="true" style="57" width="19.28515625"/>
+    <col min="6" max="6" customWidth="true" style="57" width="18.7109375"/>
+    <col min="7" max="7" customWidth="true" style="57" width="19.0"/>
+    <col min="8" max="8" customWidth="true" style="57" width="18.5703125"/>
+    <col min="9" max="9" customWidth="true" style="57" width="14.42578125"/>
+    <col min="10" max="10" customWidth="true" style="57" width="12.42578125"/>
+    <col min="11" max="16384" style="57" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="56" customFormat="1" ht="30" customHeight="1">
@@ -3932,6 +4023,198 @@
       </c>
       <c r="J1" s="56" t="s">
         <v>317</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="57">
+        <v>191</v>
+      </c>
+      <c r="B2" t="s" s="57">
+        <v>330</v>
+      </c>
+      <c r="C2" t="s" s="57">
+        <v>331</v>
+      </c>
+      <c r="D2" t="s" s="57">
+        <v>332</v>
+      </c>
+      <c r="E2" t="s" s="57">
+        <v>354</v>
+      </c>
+      <c r="F2" t="s" s="57">
+        <v>359</v>
+      </c>
+      <c r="G2" t="s" s="57">
+        <v>358</v>
+      </c>
+      <c r="H2" t="s" s="57">
+        <v>357</v>
+      </c>
+      <c r="I2" t="s" s="57">
+        <v>333</v>
+      </c>
+      <c r="J2" t="s" s="57">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="57">
+        <v>335</v>
+      </c>
+      <c r="B3" t="s" s="57">
+        <v>336</v>
+      </c>
+      <c r="C3" t="s" s="57">
+        <v>337</v>
+      </c>
+      <c r="D3" t="s" s="57">
+        <v>338</v>
+      </c>
+      <c r="E3" t="s" s="57">
+        <v>355</v>
+      </c>
+      <c r="F3" t="s" s="57">
+        <v>358</v>
+      </c>
+      <c r="G3" t="s" s="57">
+        <v>355</v>
+      </c>
+      <c r="H3" t="s" s="57">
+        <v>354</v>
+      </c>
+      <c r="I3" t="s" s="57">
+        <v>333</v>
+      </c>
+      <c r="J3" t="s" s="57">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="57">
+        <v>339</v>
+      </c>
+      <c r="B4" t="s" s="57">
+        <v>340</v>
+      </c>
+      <c r="C4" t="s" s="57">
+        <v>341</v>
+      </c>
+      <c r="D4" t="s" s="57">
+        <v>342</v>
+      </c>
+      <c r="E4" t="s" s="57">
+        <v>356</v>
+      </c>
+      <c r="F4" t="s" s="57">
+        <v>357</v>
+      </c>
+      <c r="G4" t="s" s="57">
+        <v>356</v>
+      </c>
+      <c r="H4" t="s" s="57">
+        <v>356</v>
+      </c>
+      <c r="I4" t="s" s="57">
+        <v>333</v>
+      </c>
+      <c r="J4" t="s" s="57">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="57">
+        <v>343</v>
+      </c>
+      <c r="B5" t="s" s="57">
+        <v>344</v>
+      </c>
+      <c r="C5" t="s" s="57">
+        <v>345</v>
+      </c>
+      <c r="D5" t="s" s="57">
+        <v>346</v>
+      </c>
+      <c r="E5" t="s" s="57">
+        <v>357</v>
+      </c>
+      <c r="F5" t="s" s="57">
+        <v>356</v>
+      </c>
+      <c r="G5" t="s" s="57">
+        <v>359</v>
+      </c>
+      <c r="H5" t="s" s="57">
+        <v>359</v>
+      </c>
+      <c r="I5" t="s" s="57">
+        <v>333</v>
+      </c>
+      <c r="J5" t="s" s="57">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="57">
+        <v>347</v>
+      </c>
+      <c r="B6" t="s" s="57">
+        <v>348</v>
+      </c>
+      <c r="C6" t="s" s="57">
+        <v>349</v>
+      </c>
+      <c r="D6" t="s" s="57">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s" s="57">
+        <v>358</v>
+      </c>
+      <c r="F6" t="s" s="57">
+        <v>355</v>
+      </c>
+      <c r="G6" t="s" s="57">
+        <v>354</v>
+      </c>
+      <c r="H6" t="s" s="57">
+        <v>355</v>
+      </c>
+      <c r="I6" t="s" s="57">
+        <v>333</v>
+      </c>
+      <c r="J6" t="s" s="57">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="57">
+        <v>351</v>
+      </c>
+      <c r="B7" t="s" s="57">
+        <v>340</v>
+      </c>
+      <c r="C7" t="s" s="57">
+        <v>352</v>
+      </c>
+      <c r="D7" t="s" s="57">
+        <v>353</v>
+      </c>
+      <c r="E7" t="s" s="57">
+        <v>359</v>
+      </c>
+      <c r="F7" t="s" s="57">
+        <v>354</v>
+      </c>
+      <c r="G7" t="s" s="57">
+        <v>357</v>
+      </c>
+      <c r="H7" t="s" s="57">
+        <v>358</v>
+      </c>
+      <c r="I7" t="s" s="57">
+        <v>333</v>
+      </c>
+      <c r="J7" t="s" s="57">
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -3944,10 +4227,10 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="24.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" customWidth="1"/>
-    <col min="4" max="4" width="22.5703125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="11.5703125"/>
+    <col min="2" max="2" customWidth="true" width="18.0"/>
+    <col min="3" max="3" customWidth="true" width="16.140625"/>
+    <col min="4" max="4" customWidth="true" width="22.5703125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" ht="24.75" customHeight="1">

</xml_diff>

<commit_message>
Inventory functionality is working perfectly
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -10,8 +10,8 @@
   <sheets>
     <sheet name="Test Scenarios" sheetId="1" r:id="rId1"/>
     <sheet name="Test Cases" sheetId="2" r:id="rId2"/>
-    <sheet name="Inventory" sheetId="4" r:id="rId3"/>
     <sheet name="Login" sheetId="3" r:id="rId4"/>
+    <sheet name="Inventory" r:id="rId8" sheetId="5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$2:$A$62</definedName>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="362">
   <si>
     <t>Sauce Demo Test Scenario</t>
   </si>
@@ -1137,6 +1137,12 @@
   </si>
   <si>
     <t>Test.allTheThings() T-Shirt (Red) - $15.99</t>
+  </si>
+  <si>
+    <t>02-07-2026 11:48:18</t>
+  </si>
+  <si>
+    <t>02-07-2026 11:50:56</t>
   </si>
 </sst>
 </file>
@@ -3975,253 +3981,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35697644-06C4-4BF4-833F-2719491F902D}">
-  <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" customWidth="true" style="57" width="17.42578125"/>
-    <col min="2" max="2" customWidth="true" style="57" width="18.5703125"/>
-    <col min="3" max="3" customWidth="true" style="57" width="17.42578125"/>
-    <col min="4" max="4" customWidth="true" style="57" width="16.0"/>
-    <col min="5" max="5" customWidth="true" style="57" width="19.28515625"/>
-    <col min="6" max="6" customWidth="true" style="57" width="18.7109375"/>
-    <col min="7" max="7" customWidth="true" style="57" width="19.0"/>
-    <col min="8" max="8" customWidth="true" style="57" width="18.5703125"/>
-    <col min="9" max="9" customWidth="true" style="57" width="14.42578125"/>
-    <col min="10" max="10" customWidth="true" style="57" width="12.42578125"/>
-    <col min="11" max="16384" style="57" width="9.140625"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" s="56" customFormat="1" ht="30" customHeight="1">
-      <c r="A1" s="56" t="s">
-        <v>309</v>
-      </c>
-      <c r="B1" s="56" t="s">
-        <v>310</v>
-      </c>
-      <c r="C1" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="56" t="s">
-        <v>311</v>
-      </c>
-      <c r="E1" s="56" t="s">
-        <v>312</v>
-      </c>
-      <c r="F1" s="56" t="s">
-        <v>313</v>
-      </c>
-      <c r="G1" s="56" t="s">
-        <v>314</v>
-      </c>
-      <c r="H1" s="56" t="s">
-        <v>315</v>
-      </c>
-      <c r="I1" s="56" t="s">
-        <v>316</v>
-      </c>
-      <c r="J1" s="56" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="57">
-        <v>191</v>
-      </c>
-      <c r="B2" t="s" s="57">
-        <v>330</v>
-      </c>
-      <c r="C2" t="s" s="57">
-        <v>331</v>
-      </c>
-      <c r="D2" t="s" s="57">
-        <v>332</v>
-      </c>
-      <c r="E2" t="s" s="57">
-        <v>354</v>
-      </c>
-      <c r="F2" t="s" s="57">
-        <v>359</v>
-      </c>
-      <c r="G2" t="s" s="57">
-        <v>358</v>
-      </c>
-      <c r="H2" t="s" s="57">
-        <v>357</v>
-      </c>
-      <c r="I2" t="s" s="57">
-        <v>333</v>
-      </c>
-      <c r="J2" t="s" s="57">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="57">
-        <v>335</v>
-      </c>
-      <c r="B3" t="s" s="57">
-        <v>336</v>
-      </c>
-      <c r="C3" t="s" s="57">
-        <v>337</v>
-      </c>
-      <c r="D3" t="s" s="57">
-        <v>338</v>
-      </c>
-      <c r="E3" t="s" s="57">
-        <v>355</v>
-      </c>
-      <c r="F3" t="s" s="57">
-        <v>358</v>
-      </c>
-      <c r="G3" t="s" s="57">
-        <v>355</v>
-      </c>
-      <c r="H3" t="s" s="57">
-        <v>354</v>
-      </c>
-      <c r="I3" t="s" s="57">
-        <v>333</v>
-      </c>
-      <c r="J3" t="s" s="57">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="57">
-        <v>339</v>
-      </c>
-      <c r="B4" t="s" s="57">
-        <v>340</v>
-      </c>
-      <c r="C4" t="s" s="57">
-        <v>341</v>
-      </c>
-      <c r="D4" t="s" s="57">
-        <v>342</v>
-      </c>
-      <c r="E4" t="s" s="57">
-        <v>356</v>
-      </c>
-      <c r="F4" t="s" s="57">
-        <v>357</v>
-      </c>
-      <c r="G4" t="s" s="57">
-        <v>356</v>
-      </c>
-      <c r="H4" t="s" s="57">
-        <v>356</v>
-      </c>
-      <c r="I4" t="s" s="57">
-        <v>333</v>
-      </c>
-      <c r="J4" t="s" s="57">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="57">
-        <v>343</v>
-      </c>
-      <c r="B5" t="s" s="57">
-        <v>344</v>
-      </c>
-      <c r="C5" t="s" s="57">
-        <v>345</v>
-      </c>
-      <c r="D5" t="s" s="57">
-        <v>346</v>
-      </c>
-      <c r="E5" t="s" s="57">
-        <v>357</v>
-      </c>
-      <c r="F5" t="s" s="57">
-        <v>356</v>
-      </c>
-      <c r="G5" t="s" s="57">
-        <v>359</v>
-      </c>
-      <c r="H5" t="s" s="57">
-        <v>359</v>
-      </c>
-      <c r="I5" t="s" s="57">
-        <v>333</v>
-      </c>
-      <c r="J5" t="s" s="57">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="57">
-        <v>347</v>
-      </c>
-      <c r="B6" t="s" s="57">
-        <v>348</v>
-      </c>
-      <c r="C6" t="s" s="57">
-        <v>349</v>
-      </c>
-      <c r="D6" t="s" s="57">
-        <v>350</v>
-      </c>
-      <c r="E6" t="s" s="57">
-        <v>358</v>
-      </c>
-      <c r="F6" t="s" s="57">
-        <v>355</v>
-      </c>
-      <c r="G6" t="s" s="57">
-        <v>354</v>
-      </c>
-      <c r="H6" t="s" s="57">
-        <v>355</v>
-      </c>
-      <c r="I6" t="s" s="57">
-        <v>333</v>
-      </c>
-      <c r="J6" t="s" s="57">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="57">
-        <v>351</v>
-      </c>
-      <c r="B7" t="s" s="57">
-        <v>340</v>
-      </c>
-      <c r="C7" t="s" s="57">
-        <v>352</v>
-      </c>
-      <c r="D7" t="s" s="57">
-        <v>353</v>
-      </c>
-      <c r="E7" t="s" s="57">
-        <v>359</v>
-      </c>
-      <c r="F7" t="s" s="57">
-        <v>354</v>
-      </c>
-      <c r="G7" t="s" s="57">
-        <v>357</v>
-      </c>
-      <c r="H7" t="s" s="57">
-        <v>358</v>
-      </c>
-      <c r="I7" t="s" s="57">
-        <v>333</v>
-      </c>
-      <c r="J7" t="s" s="57">
-        <v>334</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE280182-BA0C-4214-9DDE-FF3FDA9A628F}">
   <dimension ref="A1:D6"/>
@@ -4316,4 +4075,238 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>309</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>135</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>359</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>358</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>357</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>361</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>338</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>355</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>358</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>355</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="I3" t="s" s="0">
+        <v>361</v>
+      </c>
+      <c r="J3" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>339</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>340</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>341</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>342</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>356</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>357</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>356</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>356</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>361</v>
+      </c>
+      <c r="J4" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>343</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>344</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>345</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>346</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>357</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>356</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>359</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>359</v>
+      </c>
+      <c r="I5" t="s" s="0">
+        <v>361</v>
+      </c>
+      <c r="J5" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>347</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>348</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>349</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>358</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>355</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>355</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>361</v>
+      </c>
+      <c r="J6" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>351</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>340</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>352</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>353</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>359</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>357</v>
+      </c>
+      <c r="H7" t="s" s="0">
+        <v>358</v>
+      </c>
+      <c r="I7" t="s" s="0">
+        <v>361</v>
+      </c>
+      <c r="J7" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added inventory step definitions
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="363">
   <si>
     <t>Sauce Demo Test Scenario</t>
   </si>
@@ -1143,6 +1143,9 @@
   </si>
   <si>
     <t>02-07-2026 11:50:56</t>
+  </si>
+  <si>
+    <t>02-07-2026 13:37:54</t>
   </si>
 </sst>
 </file>
@@ -4140,7 +4143,7 @@
         <v>357</v>
       </c>
       <c r="I2" t="s" s="0">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J2" t="s" s="0">
         <v>334</v>
@@ -4172,7 +4175,7 @@
         <v>354</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J3" t="s" s="0">
         <v>334</v>
@@ -4204,7 +4207,7 @@
         <v>356</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J4" t="s" s="0">
         <v>334</v>
@@ -4236,7 +4239,7 @@
         <v>359</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J5" t="s" s="0">
         <v>334</v>
@@ -4268,7 +4271,7 @@
         <v>355</v>
       </c>
       <c r="I6" t="s" s="0">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J6" t="s" s="0">
         <v>334</v>
@@ -4300,7 +4303,7 @@
         <v>358</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="J7" t="s" s="0">
         <v>334</v>

</xml_diff>

<commit_message>
Logout functionality is completed
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Test Cases" sheetId="2" r:id="rId2"/>
     <sheet name="Login" sheetId="3" r:id="rId4"/>
     <sheet name="Inventory" r:id="rId8" sheetId="5"/>
+    <sheet name="Logout" r:id="rId9" sheetId="6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$2:$A$62</definedName>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="366">
   <si>
     <t>Sauce Demo Test Scenario</t>
   </si>
@@ -1146,6 +1147,15 @@
   </si>
   <si>
     <t>02-07-2026 13:37:54</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>05-07-2026 13:13:57</t>
   </si>
 </sst>
 </file>
@@ -4312,4 +4322,42 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>363</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>180</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>365</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated README.md and Allure Report
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -11,9 +11,12 @@
     <sheet name="Test Scenarios" sheetId="1" r:id="rId1"/>
     <sheet name="Test Cases" sheetId="2" r:id="rId2"/>
     <sheet name="Login" sheetId="3" r:id="rId4"/>
-    <sheet name="Inventory" r:id="rId8" sheetId="5"/>
     <sheet name="Logout" r:id="rId9" sheetId="6"/>
     <sheet name="UIValidation" r:id="rId10" sheetId="7"/>
+    <sheet name="ErrorMessages" r:id="rId11" sheetId="8"/>
+    <sheet name="Cart" r:id="rId13" sheetId="10"/>
+    <sheet name="Checkout" r:id="rId14" sheetId="11"/>
+    <sheet name="Inventory" r:id="rId12" sheetId="12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$2:$A$62</definedName>
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1449" uniqueCount="485">
   <si>
     <t>Sauce Demo Test Scenario</t>
   </si>
@@ -1262,6 +1265,258 @@
   </si>
   <si>
     <t>09-07-2026 10:52:39</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Expected Error</t>
+  </si>
+  <si>
+    <t>Actual Error</t>
+  </si>
+  <si>
+    <t>Username and password do not match any user in this service</t>
+  </si>
+  <si>
+    <t>Epic sadface: Username and password do not match any user in this service</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:00:33</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:00:39</t>
+  </si>
+  <si>
+    <t>Username is required</t>
+  </si>
+  <si>
+    <t>Epic sadface: Username is required</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:00:44</t>
+  </si>
+  <si>
+    <t>Sorry, this user has been locked out.</t>
+  </si>
+  <si>
+    <t>Epic sadface: Sorry, this user has been locked out.</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:00:50</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/assets/sauce-backpack-1200x1500-CjRW-Djj.jpg</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:01:30</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/assets/bike-light-1200x1500-DxcZRFOA.jpg</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/assets/bolt-shirt-1200x1500-mR0ldpVS.jpg</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/assets/sauce-pullover-1200x1500-BfbI-PSd.jpg</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/assets/red-onesie-1200x1500-BrSuq0ic.jpg</t>
+  </si>
+  <si>
+    <t>https://www.saucedemo.com/assets/red-tatt-1200x1500-E-qp6aYf.jpg</t>
+  </si>
+  <si>
+    <t>Product Name</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Added</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:02:30</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:02:31</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:02:55</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:02:56</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:03:25</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:03:26</t>
+  </si>
+  <si>
+    <t>First Name</t>
+  </si>
+  <si>
+    <t>Last Name</t>
+  </si>
+  <si>
+    <t>Postal Code</t>
+  </si>
+  <si>
+    <t>Error Message</t>
+  </si>
+  <si>
+    <t>Doe</t>
+  </si>
+  <si>
+    <t>560001</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>Error: First Name is required</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:04:24</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Error: Last Name is required</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:04:30</t>
+  </si>
+  <si>
+    <t>Error: Postal Code is required</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:04:37</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:05:16</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:07:16</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:07:24</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:07:29</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:07:35</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:07:40</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:10:28</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:10:29</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>09-07-2026 14:10:37</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:10:44</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:10:52</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:10:59</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:11:06</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:11:32</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:11:37</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:11:42</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:11:47</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:11:53</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:12:44</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:12:49</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:12:53</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:12:59</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:13:04</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:17:26</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:17:32</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:17:37</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:17:42</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:19:57</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:21:15</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:22:14</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:24:21</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:24:27</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:24:34</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:25:33</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:26:41</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:26:49</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:26:55</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:27:00</t>
+  </si>
+  <si>
+    <t>09-07-2026 14:27:06</t>
   </si>
 </sst>
 </file>
@@ -2691,6 +2946,398 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>421</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>422</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>423</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>424</v>
+      </c>
+      <c r="D2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>475</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>431</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>432</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>433</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>363</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>434</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="B2" s="0"/>
+      <c r="C2" t="s" s="0">
+        <v>435</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>436</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>476</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>440</v>
+      </c>
+      <c r="C3" s="0"/>
+      <c r="D3" t="s" s="0">
+        <v>436</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>477</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>169</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>440</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>435</v>
+      </c>
+      <c r="D4" s="0"/>
+      <c r="E4" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>443</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>478</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>309</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>135</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>414</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>359</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>358</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>357</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>473</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>416</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>355</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>358</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>355</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="I3" t="s" s="0">
+        <v>473</v>
+      </c>
+      <c r="J3" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>339</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>340</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>341</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>417</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>356</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>357</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>356</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>356</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>473</v>
+      </c>
+      <c r="J4" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>343</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>344</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>345</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>418</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>357</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>356</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>359</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>359</v>
+      </c>
+      <c r="I5" t="s" s="0">
+        <v>473</v>
+      </c>
+      <c r="J5" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>347</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>348</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>349</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>419</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>358</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>355</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>355</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>473</v>
+      </c>
+      <c r="J6" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>351</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>340</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>352</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>420</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>359</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>357</v>
+      </c>
+      <c r="H7" t="s" s="0">
+        <v>358</v>
+      </c>
+      <c r="I7" t="s" s="0">
+        <v>473</v>
+      </c>
+      <c r="J7" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8187F376-22C9-4E14-9441-9396C4798D74}">
   <sheetPr filterMode="1"/>
@@ -4196,240 +4843,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
-        <v>309</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s" s="0">
-        <v>311</v>
-      </c>
-      <c r="E1" t="s" s="0">
-        <v>312</v>
-      </c>
-      <c r="F1" t="s" s="0">
-        <v>313</v>
-      </c>
-      <c r="G1" t="s" s="0">
-        <v>131</v>
-      </c>
-      <c r="H1" t="s" s="0">
-        <v>135</v>
-      </c>
-      <c r="I1" t="s" s="0">
-        <v>316</v>
-      </c>
-      <c r="J1" t="s" s="0">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>191</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>330</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>331</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>332</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>354</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>359</v>
-      </c>
-      <c r="G2" t="s" s="0">
-        <v>358</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>357</v>
-      </c>
-      <c r="I2" t="s" s="0">
-        <v>362</v>
-      </c>
-      <c r="J2" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>335</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>336</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>337</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>338</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>355</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>358</v>
-      </c>
-      <c r="G3" t="s" s="0">
-        <v>355</v>
-      </c>
-      <c r="H3" t="s" s="0">
-        <v>354</v>
-      </c>
-      <c r="I3" t="s" s="0">
-        <v>362</v>
-      </c>
-      <c r="J3" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>339</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>340</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>341</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>342</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>356</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>357</v>
-      </c>
-      <c r="G4" t="s" s="0">
-        <v>356</v>
-      </c>
-      <c r="H4" t="s" s="0">
-        <v>356</v>
-      </c>
-      <c r="I4" t="s" s="0">
-        <v>362</v>
-      </c>
-      <c r="J4" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>343</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>344</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>345</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>346</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>357</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>356</v>
-      </c>
-      <c r="G5" t="s" s="0">
-        <v>359</v>
-      </c>
-      <c r="H5" t="s" s="0">
-        <v>359</v>
-      </c>
-      <c r="I5" t="s" s="0">
-        <v>362</v>
-      </c>
-      <c r="J5" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>347</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>348</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>349</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>350</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>358</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>355</v>
-      </c>
-      <c r="G6" t="s" s="0">
-        <v>354</v>
-      </c>
-      <c r="H6" t="s" s="0">
-        <v>355</v>
-      </c>
-      <c r="I6" t="s" s="0">
-        <v>362</v>
-      </c>
-      <c r="J6" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>351</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>340</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>352</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>353</v>
-      </c>
-      <c r="E7" t="s" s="0">
-        <v>359</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>354</v>
-      </c>
-      <c r="G7" t="s" s="0">
-        <v>357</v>
-      </c>
-      <c r="H7" t="s" s="0">
-        <v>358</v>
-      </c>
-      <c r="I7" t="s" s="0">
-        <v>362</v>
-      </c>
-      <c r="J7" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:D2"/>
@@ -4457,7 +4870,7 @@
         <v>364</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>365</v>
+        <v>479</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>334</v>
@@ -4470,7 +4883,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -4575,6 +4988,386 @@
         <v>334</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>385</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>446</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>366</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>447</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>368</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>448</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>254</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>370</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>449</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>372</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>450</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>385</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>464</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>366</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>465</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>368</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>466</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>254</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>370</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>467</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>372</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>468</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>385</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>480</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>366</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>481</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>368</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>482</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>254</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>370</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>483</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>372</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>484</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>401</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>402</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>403</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>363</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>404</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>405</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>469</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>404</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>405</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>470</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>408</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>409</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>471</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>411</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>412</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>472</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Ordered execution is added through multiple test runner files
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -16,8 +16,8 @@
     <sheet name="ErrorMessages" r:id="rId11" sheetId="8"/>
     <sheet name="Cart" r:id="rId13" sheetId="10"/>
     <sheet name="Checkout" r:id="rId14" sheetId="11"/>
-    <sheet name="Inventory" r:id="rId12" sheetId="12"/>
     <sheet name="SessionManagement" r:id="rId15" sheetId="13"/>
+    <sheet name="Inventory" r:id="rId16" sheetId="14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$2:$A$62</definedName>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1499" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2192" uniqueCount="560">
   <si>
     <t>Sauce Demo Test Scenario</t>
   </si>
@@ -1539,6 +1539,210 @@
   </si>
   <si>
     <t>09-07-2026 15:14:07</t>
+  </si>
+  <si>
+    <t>09-07-2026 16:41:41</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:36:58</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:37:04</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:37:09</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:37:14</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:37:19</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:40:44</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:40:51</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:40:57</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:41:03</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:41:09</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:47:20</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:47:21</t>
+  </si>
+  <si>
+    <t>Removed</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:48:03</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:48:10</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:48:37</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:48:43</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:48:49</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:48:56</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:49:02</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:50:24</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:50:30</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:50:36</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:50:41</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:50:46</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:50:51</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:50:56</t>
+  </si>
+  <si>
+    <t>10-07-2026 10:51:02</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:15:05</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:15:11</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:15:19</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:15:26</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:15:33</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:15:50</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:15:51</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:16:15</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:16:20</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:16:26</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:16:32</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:17:21</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:17:26</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:17:31</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:17:36</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:17:41</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:17:55</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:18:00</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:18:07</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:25:17</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:25:23</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:25:31</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:25:38</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:25:48</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:26:06</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:26:07</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:26:14</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:26:20</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:26:25</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:26:31</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:26:38</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:27:26</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:27:32</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:27:37</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:27:42</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:27:47</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:28:01</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:28:06</t>
+  </si>
+  <si>
+    <t>10-07-2026 11:28:11</t>
   </si>
 </sst>
 </file>
@@ -2970,7 +3174,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2991,26 +3195,6 @@
       </c>
       <c r="F1" t="s" s="0">
         <v>317</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>191</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>330</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>424</v>
-      </c>
-      <c r="D2" t="n" s="0">
-        <v>1.0</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>475</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -3020,7 +3204,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3049,84 +3233,226 @@
         <v>317</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>164</v>
-      </c>
-      <c r="B2" s="0"/>
-      <c r="C2" t="s" s="0">
-        <v>435</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>436</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>437</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>438</v>
-      </c>
-      <c r="G2" t="s" s="0">
-        <v>476</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>167</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>440</v>
-      </c>
-      <c r="C3" s="0"/>
-      <c r="D3" t="s" s="0">
-        <v>436</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>437</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>441</v>
-      </c>
-      <c r="G3" t="s" s="0">
-        <v>477</v>
-      </c>
-      <c r="H3" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>169</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>440</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>435</v>
-      </c>
-      <c r="D4" s="0"/>
-      <c r="E4" t="s" s="0">
-        <v>437</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>443</v>
-      </c>
-      <c r="G4" t="s" s="0">
-        <v>478</v>
-      </c>
-      <c r="H4" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>489</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>490</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>267</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>491</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>513</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>514</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>267</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>515</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>537</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>538</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>267</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>539</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>557</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>558</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>267</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>559</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -3189,7 +3515,7 @@
         <v>357</v>
       </c>
       <c r="I2" t="s" s="0">
-        <v>473</v>
+        <v>544</v>
       </c>
       <c r="J2" t="s" s="0">
         <v>334</v>
@@ -3221,7 +3547,7 @@
         <v>354</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>473</v>
+        <v>544</v>
       </c>
       <c r="J3" t="s" s="0">
         <v>334</v>
@@ -3253,7 +3579,7 @@
         <v>356</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>473</v>
+        <v>544</v>
       </c>
       <c r="J4" t="s" s="0">
         <v>334</v>
@@ -3285,7 +3611,7 @@
         <v>359</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>473</v>
+        <v>544</v>
       </c>
       <c r="J5" t="s" s="0">
         <v>334</v>
@@ -3317,7 +3643,7 @@
         <v>355</v>
       </c>
       <c r="I6" t="s" s="0">
-        <v>473</v>
+        <v>544</v>
       </c>
       <c r="J6" t="s" s="0">
         <v>334</v>
@@ -3349,70 +3675,9 @@
         <v>358</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>473</v>
+        <v>544</v>
       </c>
       <c r="J7" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
-        <v>260</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>261</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D1" t="s" s="0">
-        <v>489</v>
-      </c>
-      <c r="E1" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>263</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>264</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>490</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>266</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>267</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>491</v>
-      </c>
-      <c r="E3" t="s" s="0">
         <v>334</v>
       </c>
     </row>
@@ -4928,7 +5193,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -4943,20 +5208,6 @@
       </c>
       <c r="D1" t="s" s="0">
         <v>317</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>180</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>479</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -4966,7 +5217,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -4984,346 +5235,6 @@
       </c>
       <c r="E1" t="s" s="0">
         <v>317</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>244</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>385</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>396</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>247</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>366</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>397</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>250</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>368</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>398</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>254</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>370</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>399</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>256</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>372</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>400</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>244</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>385</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>446</v>
-      </c>
-      <c r="E7" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>247</v>
-      </c>
-      <c r="B8" t="s" s="0">
-        <v>366</v>
-      </c>
-      <c r="C8" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>447</v>
-      </c>
-      <c r="E8" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="0">
-        <v>250</v>
-      </c>
-      <c r="B9" t="s" s="0">
-        <v>368</v>
-      </c>
-      <c r="C9" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D9" t="s" s="0">
-        <v>448</v>
-      </c>
-      <c r="E9" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
-        <v>254</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>370</v>
-      </c>
-      <c r="C10" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>449</v>
-      </c>
-      <c r="E10" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>256</v>
-      </c>
-      <c r="B11" t="s" s="0">
-        <v>372</v>
-      </c>
-      <c r="C11" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D11" t="s" s="0">
-        <v>450</v>
-      </c>
-      <c r="E11" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="0">
-        <v>244</v>
-      </c>
-      <c r="B12" t="s" s="0">
-        <v>385</v>
-      </c>
-      <c r="C12" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D12" t="s" s="0">
-        <v>464</v>
-      </c>
-      <c r="E12" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="0">
-        <v>247</v>
-      </c>
-      <c r="B13" t="s" s="0">
-        <v>366</v>
-      </c>
-      <c r="C13" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D13" t="s" s="0">
-        <v>465</v>
-      </c>
-      <c r="E13" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="0">
-        <v>250</v>
-      </c>
-      <c r="B14" t="s" s="0">
-        <v>368</v>
-      </c>
-      <c r="C14" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D14" t="s" s="0">
-        <v>466</v>
-      </c>
-      <c r="E14" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s" s="0">
-        <v>254</v>
-      </c>
-      <c r="B15" t="s" s="0">
-        <v>370</v>
-      </c>
-      <c r="C15" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D15" t="s" s="0">
-        <v>467</v>
-      </c>
-      <c r="E15" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s" s="0">
-        <v>256</v>
-      </c>
-      <c r="B16" t="s" s="0">
-        <v>372</v>
-      </c>
-      <c r="C16" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D16" t="s" s="0">
-        <v>468</v>
-      </c>
-      <c r="E16" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s" s="0">
-        <v>244</v>
-      </c>
-      <c r="B17" t="s" s="0">
-        <v>385</v>
-      </c>
-      <c r="C17" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D17" t="s" s="0">
-        <v>480</v>
-      </c>
-      <c r="E17" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>247</v>
-      </c>
-      <c r="B18" t="s" s="0">
-        <v>366</v>
-      </c>
-      <c r="C18" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D18" t="s" s="0">
-        <v>481</v>
-      </c>
-      <c r="E18" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s" s="0">
-        <v>250</v>
-      </c>
-      <c r="B19" t="s" s="0">
-        <v>368</v>
-      </c>
-      <c r="C19" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D19" t="s" s="0">
-        <v>482</v>
-      </c>
-      <c r="E19" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s" s="0">
-        <v>254</v>
-      </c>
-      <c r="B20" t="s" s="0">
-        <v>370</v>
-      </c>
-      <c r="C20" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D20" t="s" s="0">
-        <v>483</v>
-      </c>
-      <c r="E20" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s" s="0">
-        <v>256</v>
-      </c>
-      <c r="B21" t="s" s="0">
-        <v>372</v>
-      </c>
-      <c r="C21" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="D21" t="s" s="0">
-        <v>484</v>
-      </c>
-      <c r="E21" t="s" s="0">
-        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -5333,7 +5244,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -5359,98 +5270,6 @@
         <v>317</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>224</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>228</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>404</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>405</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>485</v>
-      </c>
-      <c r="G2" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>224</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>228</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>404</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>405</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>486</v>
-      </c>
-      <c r="G3" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>229</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>228</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>408</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>409</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>487</v>
-      </c>
-      <c r="G4" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>236</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>228</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>411</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>412</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>364</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>488</v>
-      </c>
-      <c r="G5" t="s" s="0">
-        <v>334</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Added cross browser parallel execution
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2192" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3910" uniqueCount="667">
   <si>
     <t>Sauce Demo Test Scenario</t>
   </si>
@@ -1743,6 +1743,327 @@
   </si>
   <si>
     <t>10-07-2026 11:28:11</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:32:05</t>
+  </si>
+  <si>
+    <t>edge</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:32:12</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:32:18</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:32:27</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:46:12</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:46:18</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:46:23</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:46:30</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:46:37</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:46:57</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:46:58</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:47:06</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:47:13</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:47:20</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:47:27</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:47:33</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:48:26</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:48:31</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:48:36</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:48:41</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:48:47</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:49:03</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:49:09</t>
+  </si>
+  <si>
+    <t>11-07-2026 12:49:15</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:05:43</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:06:54</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:06:55</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:08:13</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:08:14</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:12:56</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:13:03</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:13:10</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:13:17</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:14:02</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:14:09</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:14:15</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:14:21</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:20:07</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:20:14</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:20:15</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:20:24</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:20:34</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:33:47</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:33:48</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:33:57</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:34:06</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:34:15</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:45:58</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:46:05</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:46:09</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:46:11</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:46:17</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:46:18</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:46:24</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:57:33</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:57:42</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:57:49</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:57:52</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:57:56</t>
+  </si>
+  <si>
+    <t>11-07-2026 13:58:10</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:54:06</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:54:11</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:54:14</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:54:21</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:54:24</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:54:30</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:54:34</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:54:37</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:54:46</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:54:51</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:55:14</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:55:15</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:55:16</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:55:24</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:55:25</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:55:27</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:55:38</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:55:50</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:56:01</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:56:02</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:56:13</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:56:27</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:57:38</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:57:46</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:57:54</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:58:00</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:58:03</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:58:10</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:58:12</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:58:19</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:58:29</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:58:33</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:58:39</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:58:44</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:59:00</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:59:07</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:59:13</t>
+  </si>
+  <si>
+    <t>11-07-2026 14:59:20</t>
+  </si>
+  <si>
+    <t>11-07-2026 15:36:45</t>
+  </si>
+  <si>
+    <t>11-07-2026 15:36:46</t>
+  </si>
+  <si>
+    <t>11-07-2026 15:47:56</t>
+  </si>
+  <si>
+    <t>11-07-2026 15:47:57</t>
+  </si>
+  <si>
+    <t>11-07-2026 15:54:11</t>
+  </si>
+  <si>
+    <t>11-07-2026 16:00:37</t>
+  </si>
+  <si>
+    <t>11-07-2026 16:00:38</t>
+  </si>
+  <si>
+    <t>11-07-2026 17:08:28</t>
   </si>
 </sst>
 </file>
@@ -1750,7 +2071,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1804,8 +2125,53 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
+      <b val="true"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1818,8 +2184,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="42"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="42"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -1996,11 +2372,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin"/>
+    </border>
+    <border>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2170,6 +2564,57 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="19" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="19" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="19" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyAlignment="true" applyBorder="true">
+      <alignment wrapText="true" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyAlignment="true" applyBorder="true">
+      <alignment wrapText="true" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="19" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="19" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyAlignment="true" applyBorder="true">
+      <alignment wrapText="true" vertical="center" horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyAlignment="true" applyBorder="true">
+      <alignment wrapText="true" vertical="center" horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="19" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="19" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyAlignment="true" applyBorder="true">
+      <alignment wrapText="false" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyAlignment="true" applyBorder="true">
+      <alignment wrapText="false" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="19" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="19" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyAlignment="true" applyBorder="true">
+      <alignment wrapText="false" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyAlignment="true" applyBorder="true">
+      <alignment wrapText="false" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3174,7 +3619,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3195,6 +3640,166 @@
       </c>
       <c r="F1" t="s" s="0">
         <v>317</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>424</v>
+      </c>
+      <c r="D2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>631</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>424</v>
+      </c>
+      <c r="D3" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>632</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>424</v>
+      </c>
+      <c r="D4" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>632</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>505</v>
+      </c>
+      <c r="D5" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>633</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>424</v>
+      </c>
+      <c r="D6" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>634</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>424</v>
+      </c>
+      <c r="D7" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>635</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>424</v>
+      </c>
+      <c r="D8" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>635</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>505</v>
+      </c>
+      <c r="D9" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>635</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -3204,7 +3809,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3231,6 +3836,202 @@
       </c>
       <c r="H1" t="s" s="0">
         <v>317</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>440</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>435</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>436</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>453</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>636</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>440</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>435</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>436</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>453</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>637</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="B4" s="0"/>
+      <c r="C4" t="s" s="0">
+        <v>435</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>436</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>637</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>440</v>
+      </c>
+      <c r="C5" s="0"/>
+      <c r="D5" t="s" s="0">
+        <v>436</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>638</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="B6" s="0"/>
+      <c r="C6" t="s" s="0">
+        <v>435</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>436</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>638</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>440</v>
+      </c>
+      <c r="C7" s="0"/>
+      <c r="D7" t="s" s="0">
+        <v>436</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>639</v>
+      </c>
+      <c r="H7" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>169</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>440</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>435</v>
+      </c>
+      <c r="D8" s="0"/>
+      <c r="E8" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>443</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>640</v>
+      </c>
+      <c r="H8" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>169</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>440</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>435</v>
+      </c>
+      <c r="D9" s="0"/>
+      <c r="E9" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>443</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>641</v>
+      </c>
+      <c r="H9" t="s" s="0">
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -3240,7 +4041,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3444,6 +4245,159 @@
         <v>559</v>
       </c>
       <c r="E12" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>582</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>583</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>267</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>584</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>652</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>654</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>267</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>655</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>656</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>657</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>267</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>658</v>
+      </c>
+      <c r="E21" t="s" s="0">
         <v>334</v>
       </c>
     </row>
@@ -3456,50 +4410,62 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="30.0"/>
+    <col min="2" max="2" customWidth="true" width="12.0"/>
+    <col min="3" max="3" customWidth="true" width="80.0"/>
+    <col min="4" max="4" customWidth="true" width="40.0"/>
+    <col min="5" max="5" customWidth="true" width="35.0"/>
+    <col min="6" max="6" customWidth="true" width="35.0"/>
+    <col min="7" max="7" customWidth="true" width="35.0"/>
+    <col min="8" max="8" customWidth="true" width="35.0"/>
+    <col min="9" max="9" customWidth="true" width="25.0"/>
+    <col min="10" max="10" customWidth="true" width="12.0"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
+    <row r="1" ht="25.0" customHeight="true">
+      <c r="A1" t="s" s="72">
         <v>309</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s" s="72">
         <v>310</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s" s="72">
         <v>3</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s" s="72">
         <v>311</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s" s="72">
         <v>312</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s" s="72">
         <v>313</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s" s="72">
         <v>131</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s" s="72">
         <v>135</v>
       </c>
-      <c r="I1" t="s" s="0">
+      <c r="I1" t="s" s="72">
         <v>316</v>
       </c>
-      <c r="J1" t="s" s="0">
+      <c r="J1" t="s" s="72">
         <v>317</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
+    <row r="2" ht="30.0" customHeight="true">
+      <c r="A2" t="s" s="74">
         <v>191</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s" s="74">
         <v>330</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s" s="74">
         <v>331</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s" s="74">
         <v>414</v>
       </c>
       <c r="E2" t="s" s="0">
@@ -3514,24 +4480,24 @@
       <c r="H2" t="s" s="0">
         <v>357</v>
       </c>
-      <c r="I2" t="s" s="0">
-        <v>544</v>
-      </c>
-      <c r="J2" t="s" s="0">
+      <c r="I2" t="s" s="74">
+        <v>666</v>
+      </c>
+      <c r="J2" t="s" s="74">
         <v>334</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
+    <row r="3" ht="30.0" customHeight="true">
+      <c r="A3" t="s" s="74">
         <v>335</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s" s="74">
         <v>336</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s" s="74">
         <v>337</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s" s="74">
         <v>416</v>
       </c>
       <c r="E3" t="s" s="0">
@@ -3546,24 +4512,24 @@
       <c r="H3" t="s" s="0">
         <v>354</v>
       </c>
-      <c r="I3" t="s" s="0">
-        <v>544</v>
-      </c>
-      <c r="J3" t="s" s="0">
+      <c r="I3" t="s" s="74">
+        <v>666</v>
+      </c>
+      <c r="J3" t="s" s="74">
         <v>334</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
+    <row r="4" ht="30.0" customHeight="true">
+      <c r="A4" t="s" s="74">
         <v>339</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s" s="74">
         <v>340</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="C4" t="s" s="74">
         <v>341</v>
       </c>
-      <c r="D4" t="s" s="0">
+      <c r="D4" t="s" s="74">
         <v>417</v>
       </c>
       <c r="E4" t="s" s="0">
@@ -3578,24 +4544,24 @@
       <c r="H4" t="s" s="0">
         <v>356</v>
       </c>
-      <c r="I4" t="s" s="0">
-        <v>544</v>
-      </c>
-      <c r="J4" t="s" s="0">
+      <c r="I4" t="s" s="74">
+        <v>666</v>
+      </c>
+      <c r="J4" t="s" s="74">
         <v>334</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
+    <row r="5" ht="30.0" customHeight="true">
+      <c r="A5" t="s" s="74">
         <v>343</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s" s="74">
         <v>344</v>
       </c>
-      <c r="C5" t="s" s="0">
+      <c r="C5" t="s" s="74">
         <v>345</v>
       </c>
-      <c r="D5" t="s" s="0">
+      <c r="D5" t="s" s="74">
         <v>418</v>
       </c>
       <c r="E5" t="s" s="0">
@@ -3610,24 +4576,24 @@
       <c r="H5" t="s" s="0">
         <v>359</v>
       </c>
-      <c r="I5" t="s" s="0">
-        <v>544</v>
-      </c>
-      <c r="J5" t="s" s="0">
+      <c r="I5" t="s" s="74">
+        <v>666</v>
+      </c>
+      <c r="J5" t="s" s="74">
         <v>334</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
+    <row r="6" ht="30.0" customHeight="true">
+      <c r="A6" t="s" s="74">
         <v>347</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s" s="74">
         <v>348</v>
       </c>
-      <c r="C6" t="s" s="0">
+      <c r="C6" t="s" s="74">
         <v>349</v>
       </c>
-      <c r="D6" t="s" s="0">
+      <c r="D6" t="s" s="74">
         <v>419</v>
       </c>
       <c r="E6" t="s" s="0">
@@ -3642,24 +4608,24 @@
       <c r="H6" t="s" s="0">
         <v>355</v>
       </c>
-      <c r="I6" t="s" s="0">
-        <v>544</v>
-      </c>
-      <c r="J6" t="s" s="0">
+      <c r="I6" t="s" s="74">
+        <v>666</v>
+      </c>
+      <c r="J6" t="s" s="74">
         <v>334</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
+    <row r="7" ht="30.0" customHeight="true">
+      <c r="A7" t="s" s="74">
         <v>351</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" t="s" s="74">
         <v>340</v>
       </c>
-      <c r="C7" t="s" s="0">
+      <c r="C7" t="s" s="74">
         <v>352</v>
       </c>
-      <c r="D7" t="s" s="0">
+      <c r="D7" t="s" s="74">
         <v>420</v>
       </c>
       <c r="E7" t="s" s="0">
@@ -3674,10 +4640,10 @@
       <c r="H7" t="s" s="0">
         <v>358</v>
       </c>
-      <c r="I7" t="s" s="0">
-        <v>544</v>
-      </c>
-      <c r="J7" t="s" s="0">
+      <c r="I7" t="s" s="74">
+        <v>666</v>
+      </c>
+      <c r="J7" t="s" s="74">
         <v>334</v>
       </c>
     </row>
@@ -5193,7 +6159,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -5208,6 +6174,20 @@
       </c>
       <c r="D1" t="s" s="0">
         <v>317</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>180</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>642</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -5217,7 +6197,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -5235,6 +6215,176 @@
       </c>
       <c r="E1" t="s" s="0">
         <v>317</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>385</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>643</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>366</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>644</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>368</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>645</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>385</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>646</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>254</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>370</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>647</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>366</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>648</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>372</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>649</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>368</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>650</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>254</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>370</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>651</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>372</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>653</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -5244,7 +6394,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -5270,6 +6420,190 @@
         <v>317</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>404</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>405</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>621</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>404</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>405</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>622</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>404</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>405</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>623</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>404</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>405</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>624</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>408</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>409</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>625</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>408</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>409</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>626</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>411</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>412</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>627</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>411</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>412</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>364</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>628</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>334</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>